<commit_message>
Publiceer De Vijf Ontwikkelingsassen: NL/DE/EN artikel + hero + xlsx rijen X.15.11 onder Onderzoek
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR2336"/>
+  <dimension ref="B2:AR2339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -96907,6 +96907,285 @@
         </is>
       </c>
     </row>
+    <row r="2337">
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>1.15.11</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="D2337" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2337" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2337" t="inlineStr">
+        <is>
+          <t>De Vijf Ontwikkelingsassen — Kernuitwerking</t>
+        </is>
+      </c>
+      <c r="G2337" t="inlineStr">
+        <is>
+          <t>Van oplossingen naar rekenwerk — deelrapport voor beleidsvorming</t>
+        </is>
+      </c>
+      <c r="H2337" t="inlineStr">
+        <is>
+          <t>Zeven interventiescenarios voor vier gelijktijdige verlieslagen: opvoedingscrisis, AI-arbeidsmarkt, industrie-afbouw en talent-uitstroom. Nederlandse Renaissance levert +€1.480 mld tot 2075, break-even 2050. Berekend met neuraal invloedsmodel (R² 0,75-1,00).</t>
+        </is>
+      </c>
+      <c r="I2337" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+        </is>
+      </c>
+      <c r="J2337" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+        </is>
+      </c>
+      <c r="K2337" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2337" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2337" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2337" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2337" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2337" t="n">
+        <v>11</v>
+      </c>
+      <c r="T2337" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2337" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+        </is>
+      </c>
+      <c r="AK2337" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2337" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="B2338" t="inlineStr">
+        <is>
+          <t>2.15.11</t>
+        </is>
+      </c>
+      <c r="C2338" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="D2338" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2338" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2338" t="inlineStr">
+        <is>
+          <t>Die Fünf Entwicklungsachsen — Kernausarbeitung</t>
+        </is>
+      </c>
+      <c r="G2338" t="inlineStr">
+        <is>
+          <t>Von Lösungen zur Modellrechnung — Teilbericht zur Politikgestaltung</t>
+        </is>
+      </c>
+      <c r="H2338" t="inlineStr">
+        <is>
+          <t>Sieben Interventionsszenarien für vier gleichzeitige Verlustphasen: Erziehungskrise, KI-Arbeitsmarkt, Deindustrialisierung und Talentabwanderung. Niederländische Renaissance liefert +€1.480 Mrd bis 2075, Break-even 2050. Berechnet mit neuronalem Einflussmodell (R² 0,75-1,00).</t>
+        </is>
+      </c>
+      <c r="I2338" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+        </is>
+      </c>
+      <c r="J2338" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+        </is>
+      </c>
+      <c r="K2338" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2338" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2338" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2338" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2338" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2338" t="n">
+        <v>11</v>
+      </c>
+      <c r="T2338" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2338" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+        </is>
+      </c>
+      <c r="AK2338" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2338" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>3.15.11</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="D2339" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2339" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2339" t="inlineStr">
+        <is>
+          <t>The Five Development Axes — Core Elaboration</t>
+        </is>
+      </c>
+      <c r="G2339" t="inlineStr">
+        <is>
+          <t>From solutions to modelling — subreport for policy formation</t>
+        </is>
+      </c>
+      <c r="H2339" t="inlineStr">
+        <is>
+          <t>Seven intervention scenarios for four simultaneous loss episodes: parenting crisis, AI labour market, industrial decline and talent outflow. Dutch Renaissance delivers +€1,480 bn by 2075, break-even 2050. Computed with neural influence model (R² 0.75-1.00).</t>
+        </is>
+      </c>
+      <c r="I2339" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+        </is>
+      </c>
+      <c r="J2339" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+        </is>
+      </c>
+      <c r="K2339" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2339" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2339" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2339" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2339" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2339" t="n">
+        <v>11</v>
+      </c>
+      <c r="T2339" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2339" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+        </is>
+      </c>
+      <c r="AK2339" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2339" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publiceer volledig rapport Vijf Ontwikkelingsassen v29: NL/DE/EN + 114 grafieken + hero + xlsx X.15.12 met kleuren per Deel
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2339"/>
+  <dimension ref="B2:AR2342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -97186,6 +97186,285 @@
         </is>
       </c>
     </row>
+    <row r="2340">
+      <c r="B2340" t="inlineStr">
+        <is>
+          <t>1.15.12</t>
+        </is>
+      </c>
+      <c r="C2340" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="D2340" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2340" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2340" t="inlineStr">
+        <is>
+          <t>De Vijf Ontwikkelingsassen — Volledig rapport (v29)</t>
+        </is>
+      </c>
+      <c r="G2340" t="inlineStr">
+        <is>
+          <t>Lichaam, gevoel, aandacht, taal en gevoelsblindheid — 114 grafieken</t>
+        </is>
+      </c>
+      <c r="H2340" t="inlineStr">
+        <is>
+          <t>Integrale analyse van vier verlieslagen die Nederland gelijktijdig raken: opvoedingscrisis, AI-arbeidsmarkttransitie, industrie-afbouw en talent-uitstroom. 114 grafieken met volledige beschrijving, methode en bron. Het volledige rapport waarop de kortere kernuitwerking is gebaseerd.</t>
+        </is>
+      </c>
+      <c r="I2340" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
+        </is>
+      </c>
+      <c r="J2340" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
+        </is>
+      </c>
+      <c r="K2340" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2340" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2340" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2340" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2340" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2340" t="n">
+        <v>12</v>
+      </c>
+      <c r="T2340" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2340" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
+        </is>
+      </c>
+      <c r="AK2340" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2340" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="B2341" t="inlineStr">
+        <is>
+          <t>2.15.12</t>
+        </is>
+      </c>
+      <c r="C2341" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="D2341" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2341" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2341" t="inlineStr">
+        <is>
+          <t>Die Fünf Entwicklungsachsen — Vollständiger Bericht (v29)</t>
+        </is>
+      </c>
+      <c r="G2341" t="inlineStr">
+        <is>
+          <t>Körper, Gefühl, Aufmerksamkeit, Sprache und Gefühlsblindheit — 114 Grafiken</t>
+        </is>
+      </c>
+      <c r="H2341" t="inlineStr">
+        <is>
+          <t>Integrale Analyse von vier Verlustphasen, die die Niederlande gleichzeitig betreffen: Erziehungskrise, KI-Arbeitsmarktwandel, Deindustrialisierung und Talentabwanderung. 114 Grafiken mit vollständiger Beschreibung, Methode und Quelle.</t>
+        </is>
+      </c>
+      <c r="I2341" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
+        </is>
+      </c>
+      <c r="J2341" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
+        </is>
+      </c>
+      <c r="K2341" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2341" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2341" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2341" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2341" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2341" t="n">
+        <v>12</v>
+      </c>
+      <c r="T2341" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2341" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
+        </is>
+      </c>
+      <c r="AK2341" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2341" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="B2342" t="inlineStr">
+        <is>
+          <t>3.15.12</t>
+        </is>
+      </c>
+      <c r="C2342" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="D2342" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2342" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2342" t="inlineStr">
+        <is>
+          <t>The Five Development Axes — Full Report (v29)</t>
+        </is>
+      </c>
+      <c r="G2342" t="inlineStr">
+        <is>
+          <t>Body, feeling, attention, language and sensory blindness — 114 graphs</t>
+        </is>
+      </c>
+      <c r="H2342" t="inlineStr">
+        <is>
+          <t>Integrated analysis of four loss episodes hitting the Netherlands simultaneously: parenting crisis, AI labour market transition, industrial decline and talent outflow. 114 graphs with full description, methodology and sources.</t>
+        </is>
+      </c>
+      <c r="I2342" t="inlineStr">
+        <is>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
+        </is>
+      </c>
+      <c r="J2342" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
+        </is>
+      </c>
+      <c r="K2342" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L2342" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M2342" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N2342" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R2342" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2342" t="n">
+        <v>12</v>
+      </c>
+      <c r="T2342" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2342" t="inlineStr">
+        <is>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
+        </is>
+      </c>
+      <c r="AK2342" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="AL2342" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Verwijder Vijf Ontwikkelingsassen — Kernuitwerking (NL/DE/EN, .15.11) — user wil terugkomen met nieuw artikel
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2342"/>
+  <dimension ref="A2:AR2339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -96910,7 +96910,7 @@
     <row r="2337">
       <c r="B2337" t="inlineStr">
         <is>
-          <t>1.15.11</t>
+          <t>1.15.12</t>
         </is>
       </c>
       <c r="C2337" t="inlineStr">
@@ -96930,27 +96930,27 @@
       </c>
       <c r="F2337" t="inlineStr">
         <is>
-          <t>De Vijf Ontwikkelingsassen — Kernuitwerking</t>
+          <t>De Vijf Ontwikkelingsassen — Volledig rapport (v29)</t>
         </is>
       </c>
       <c r="G2337" t="inlineStr">
         <is>
-          <t>Van oplossingen naar rekenwerk — deelrapport voor beleidsvorming</t>
+          <t>Lichaam, gevoel, aandacht, taal en gevoelsblindheid — 114 grafieken</t>
         </is>
       </c>
       <c r="H2337" t="inlineStr">
         <is>
-          <t>Zeven interventiescenarios voor vier gelijktijdige verlieslagen: opvoedingscrisis, AI-arbeidsmarkt, industrie-afbouw en talent-uitstroom. Nederlandse Renaissance levert +€1.480 mld tot 2075, break-even 2050. Berekend met neuraal invloedsmodel (R² 0,75-1,00).</t>
+          <t>Integrale analyse van vier verlieslagen die Nederland gelijktijdig raken: opvoedingscrisis, AI-arbeidsmarkttransitie, industrie-afbouw en talent-uitstroom. 114 grafieken met volledige beschrijving, methode en bron. Het volledige rapport waarop de kortere kernuitwerking is gebaseerd.</t>
         </is>
       </c>
       <c r="I2337" t="inlineStr">
         <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
         </is>
       </c>
       <c r="J2337" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
         </is>
       </c>
       <c r="K2337" t="inlineStr">
@@ -96979,14 +96979,14 @@
         </is>
       </c>
       <c r="S2337" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T2337" t="b">
         <v>1</v>
       </c>
       <c r="AI2337" t="inlineStr">
         <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
         </is>
       </c>
       <c r="AK2337" t="inlineStr">
@@ -97003,7 +97003,7 @@
     <row r="2338">
       <c r="B2338" t="inlineStr">
         <is>
-          <t>2.15.11</t>
+          <t>2.15.12</t>
         </is>
       </c>
       <c r="C2338" t="inlineStr">
@@ -97023,27 +97023,27 @@
       </c>
       <c r="F2338" t="inlineStr">
         <is>
-          <t>Die Fünf Entwicklungsachsen — Kernausarbeitung</t>
+          <t>Die Fünf Entwicklungsachsen — Vollständiger Bericht (v29)</t>
         </is>
       </c>
       <c r="G2338" t="inlineStr">
         <is>
-          <t>Von Lösungen zur Modellrechnung — Teilbericht zur Politikgestaltung</t>
+          <t>Körper, Gefühl, Aufmerksamkeit, Sprache und Gefühlsblindheit — 114 Grafiken</t>
         </is>
       </c>
       <c r="H2338" t="inlineStr">
         <is>
-          <t>Sieben Interventionsszenarien für vier gleichzeitige Verlustphasen: Erziehungskrise, KI-Arbeitsmarkt, Deindustrialisierung und Talentabwanderung. Niederländische Renaissance liefert +€1.480 Mrd bis 2075, Break-even 2050. Berechnet mit neuronalem Einflussmodell (R² 0,75-1,00).</t>
+          <t>Integrale Analyse von vier Verlustphasen, die die Niederlande gleichzeitig betreffen: Erziehungskrise, KI-Arbeitsmarktwandel, Deindustrialisierung und Talentabwanderung. 114 Grafiken mit vollständiger Beschreibung, Methode und Quelle.</t>
         </is>
       </c>
       <c r="I2338" t="inlineStr">
         <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
         </is>
       </c>
       <c r="J2338" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
         </is>
       </c>
       <c r="K2338" t="inlineStr">
@@ -97072,14 +97072,14 @@
         </is>
       </c>
       <c r="S2338" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T2338" t="b">
         <v>1</v>
       </c>
       <c r="AI2338" t="inlineStr">
         <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
         </is>
       </c>
       <c r="AK2338" t="inlineStr">
@@ -97096,7 +97096,7 @@
     <row r="2339">
       <c r="B2339" t="inlineStr">
         <is>
-          <t>3.15.11</t>
+          <t>3.15.12</t>
         </is>
       </c>
       <c r="C2339" t="inlineStr">
@@ -97116,27 +97116,27 @@
       </c>
       <c r="F2339" t="inlineStr">
         <is>
-          <t>The Five Development Axes — Core Elaboration</t>
+          <t>The Five Development Axes — Full Report (v29)</t>
         </is>
       </c>
       <c r="G2339" t="inlineStr">
         <is>
-          <t>From solutions to modelling — subreport for policy formation</t>
+          <t>Body, feeling, attention, language and sensory blindness — 114 graphs</t>
         </is>
       </c>
       <c r="H2339" t="inlineStr">
         <is>
-          <t>Seven intervention scenarios for four simultaneous loss episodes: parenting crisis, AI labour market, industrial decline and talent outflow. Dutch Renaissance delivers +€1,480 bn by 2075, break-even 2050. Computed with neural influence model (R² 0.75-1.00).</t>
+          <t>Integrated analysis of four loss episodes hitting the Netherlands simultaneously: parenting crisis, AI labour market transition, industrial decline and talent outflow. 114 graphs with full description, methodology and sources.</t>
         </is>
       </c>
       <c r="I2339" t="inlineStr">
         <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen.html</t>
+          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
         </is>
       </c>
       <c r="J2339" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen.jpg</t>
+          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
         </is>
       </c>
       <c r="K2339" t="inlineStr">
@@ -97165,14 +97165,14 @@
         </is>
       </c>
       <c r="S2339" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T2339" t="b">
         <v>1</v>
       </c>
       <c r="AI2339" t="inlineStr">
         <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance</t>
+          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
         </is>
       </c>
       <c r="AK2339" t="inlineStr">
@@ -97181,285 +97181,6 @@
         </is>
       </c>
       <c r="AL2339" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-    </row>
-    <row r="2340">
-      <c r="B2340" t="inlineStr">
-        <is>
-          <t>1.15.12</t>
-        </is>
-      </c>
-      <c r="C2340" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="D2340" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E2340" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F2340" t="inlineStr">
-        <is>
-          <t>De Vijf Ontwikkelingsassen — Volledig rapport (v29)</t>
-        </is>
-      </c>
-      <c r="G2340" t="inlineStr">
-        <is>
-          <t>Lichaam, gevoel, aandacht, taal en gevoelsblindheid — 114 grafieken</t>
-        </is>
-      </c>
-      <c r="H2340" t="inlineStr">
-        <is>
-          <t>Integrale analyse van vier verlieslagen die Nederland gelijktijdig raken: opvoedingscrisis, AI-arbeidsmarkttransitie, industrie-afbouw en talent-uitstroom. 114 grafieken met volledige beschrijving, methode en bron. Het volledige rapport waarop de kortere kernuitwerking is gebaseerd.</t>
-        </is>
-      </c>
-      <c r="I2340" t="inlineStr">
-        <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
-        </is>
-      </c>
-      <c r="J2340" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
-        </is>
-      </c>
-      <c r="K2340" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L2340" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M2340" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N2340" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="R2340" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S2340" t="n">
-        <v>12</v>
-      </c>
-      <c r="T2340" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI2340" t="inlineStr">
-        <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
-        </is>
-      </c>
-      <c r="AK2340" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="AL2340" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-    </row>
-    <row r="2341">
-      <c r="B2341" t="inlineStr">
-        <is>
-          <t>2.15.12</t>
-        </is>
-      </c>
-      <c r="C2341" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
-      </c>
-      <c r="D2341" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="E2341" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F2341" t="inlineStr">
-        <is>
-          <t>Die Fünf Entwicklungsachsen — Vollständiger Bericht (v29)</t>
-        </is>
-      </c>
-      <c r="G2341" t="inlineStr">
-        <is>
-          <t>Körper, Gefühl, Aufmerksamkeit, Sprache und Gefühlsblindheit — 114 Grafiken</t>
-        </is>
-      </c>
-      <c r="H2341" t="inlineStr">
-        <is>
-          <t>Integrale Analyse von vier Verlustphasen, die die Niederlande gleichzeitig betreffen: Erziehungskrise, KI-Arbeitsmarktwandel, Deindustrialisierung und Talentabwanderung. 114 Grafiken mit vollständiger Beschreibung, Methode und Quelle.</t>
-        </is>
-      </c>
-      <c r="I2341" t="inlineStr">
-        <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
-        </is>
-      </c>
-      <c r="J2341" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
-        </is>
-      </c>
-      <c r="K2341" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L2341" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M2341" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N2341" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="R2341" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S2341" t="n">
-        <v>12</v>
-      </c>
-      <c r="T2341" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI2341" t="inlineStr">
-        <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
-        </is>
-      </c>
-      <c r="AK2341" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="AL2341" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-    </row>
-    <row r="2342">
-      <c r="B2342" t="inlineStr">
-        <is>
-          <t>3.15.12</t>
-        </is>
-      </c>
-      <c r="C2342" t="inlineStr">
-        <is>
-          <t>3.15</t>
-        </is>
-      </c>
-      <c r="D2342" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E2342" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F2342" t="inlineStr">
-        <is>
-          <t>The Five Development Axes — Full Report (v29)</t>
-        </is>
-      </c>
-      <c r="G2342" t="inlineStr">
-        <is>
-          <t>Body, feeling, attention, language and sensory blindness — 114 graphs</t>
-        </is>
-      </c>
-      <c r="H2342" t="inlineStr">
-        <is>
-          <t>Integrated analysis of four loss episodes hitting the Netherlands simultaneously: parenting crisis, AI labour market transition, industrial decline and talent outflow. 114 graphs with full description, methodology and sources.</t>
-        </is>
-      </c>
-      <c r="I2342" t="inlineStr">
-        <is>
-          <t>wat-opkomt/vijf-ontwikkelingsassen-volledig.html</t>
-        </is>
-      </c>
-      <c r="J2342" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_vijf-ontwikkelingsassen-volledig.jpg</t>
-        </is>
-      </c>
-      <c r="K2342" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L2342" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M2342" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N2342" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="R2342" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S2342" t="n">
-        <v>12</v>
-      </c>
-      <c r="T2342" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI2342" t="inlineStr">
-        <is>
-          <t>onderzoek, opvoeding, beleid, rekenmodel, PISA, WIA, Nederlandse Renaissance, volledig rapport</t>
-        </is>
-      </c>
-      <c r="AK2342" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="AL2342" t="inlineStr">
         <is>
           <t>Jacobus van Merksteijn</t>
         </is>

</xml_diff>